<commit_message>
Complete frequency and severity model evaluation
</commit_message>
<xml_diff>
--- a/docs/Zeiterfassung_Abschlussprojekt.xlsx
+++ b/docs/Zeiterfassung_Abschlussprojekt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mesut\Desktop\kfz-insurance-risk-platform\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E6E6AB-91D4-4957-8B4F-07EB29E7915A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{846658C4-2EEF-4601-AC11-63087F5E43D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zeiterfassung" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="67">
   <si>
     <t>Zeiterfassung Abschlussprojekt — Mesut Karagöz</t>
   </si>
@@ -208,6 +208,36 @@
   </si>
   <si>
     <t>Bewerbungen  vorbereitet und versendet</t>
+  </si>
+  <si>
+    <t>Severity-Aggregation und fachliche Bereinigungsentscheidungen umgesetzt</t>
+  </si>
+  <si>
+    <t>Bewerbungen vorbereitet und versendet</t>
+  </si>
+  <si>
+    <t>Curated Layer erstellt und Data-Quality-Regeln technisch umgesetzt</t>
+  </si>
+  <si>
+    <t>Feature Engineering durchgeführt und Curated-Datensatz validiert</t>
+  </si>
+  <si>
+    <t>PostgreSQL-Kerntabellen aufgebaut und Daten über Python geladen</t>
+  </si>
+  <si>
+    <t>Analytische Views, SQL-Prüfungen und Data-Quality-Dokumentation abgeschlossen</t>
+  </si>
+  <si>
+    <t>Datenbereinigung</t>
+  </si>
+  <si>
+    <t>Feature Engineering</t>
+  </si>
+  <si>
+    <t>SQL-Datenmodell</t>
+  </si>
+  <si>
+    <t>Validierung und Dokumentation</t>
   </si>
 </sst>
 </file>
@@ -230,65 +260,65 @@
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF5F5E5A"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF5F5E5A"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF993C1D"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF5F5E5A"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF854F0B"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -409,12 +439,12 @@
     <xf numFmtId="165" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -685,80 +715,80 @@
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="7" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="46" customWidth="1"/>
+    <col min="4" max="4" width="106.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="49.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -991,114 +1021,214 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
-      <c r="B20" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="8"/>
+      <c r="A20" s="2">
+        <v>46251</v>
+      </c>
+      <c r="B20" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="5">
+        <v>5</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
-      <c r="B21" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="8"/>
+      <c r="A21" s="2">
+        <v>46251</v>
+      </c>
+      <c r="B21" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="5">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="7"/>
-      <c r="B22" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="8"/>
+      <c r="A22" s="2">
+        <v>46252</v>
+      </c>
+      <c r="B22" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" s="5">
+        <v>5</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="7"/>
-      <c r="B23" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="8"/>
+      <c r="A23" s="2">
+        <v>46252</v>
+      </c>
+      <c r="B23" s="3">
+        <f>IF(A23="","",WEEKNUM(A23,2))</f>
+        <v>34</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="5">
+        <v>2</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="7"/>
-      <c r="B24" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="8"/>
+      <c r="A24" s="2">
+        <v>46253</v>
+      </c>
+      <c r="B24" s="3">
+        <f>IF(A24="","",WEEKNUM(A24,2))</f>
+        <v>34</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="5">
+        <v>4</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="7"/>
-      <c r="B25" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="8"/>
+      <c r="A25" s="2">
+        <v>46253</v>
+      </c>
+      <c r="B25" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E25" s="5">
+        <v>3</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="7"/>
-      <c r="B26" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="8"/>
+      <c r="A26" s="2">
+        <v>46254</v>
+      </c>
+      <c r="B26" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="5">
+        <v>4</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="7"/>
-      <c r="B27" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="8"/>
+      <c r="A27" s="2">
+        <v>46254</v>
+      </c>
+      <c r="B27" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" s="5">
+        <v>3</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="7"/>
-      <c r="B28" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="8"/>
+      <c r="A28" s="2">
+        <v>46255</v>
+      </c>
+      <c r="B28" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="5">
+        <v>5</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="7"/>
-      <c r="B29" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="8"/>
+      <c r="A29" s="2">
+        <v>46255</v>
+      </c>
+      <c r="B29" s="3">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E29" s="5">
+        <v>2</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
@@ -4391,24 +4521,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
@@ -4511,15 +4641,15 @@
       </c>
       <c r="D8" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A8,Zeiterfassung!$C$11:$C$325,"Abschlussprojekt")</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E8" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A8,Zeiterfassung!$C$11:$C$325,"Bewerbungen")</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F8" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -4668,36 +4798,36 @@
       </c>
       <c r="D15" s="25">
         <f>SUM(D5:D14)</f>
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="E15" s="25">
         <f>SUM(E5:E14)</f>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F15" s="25">
         <f>SUM(F5:F14)</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="27" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Add Tweedie challenger and model comparison
</commit_message>
<xml_diff>
--- a/docs/Zeiterfassung_Abschlussprojekt.xlsx
+++ b/docs/Zeiterfassung_Abschlussprojekt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mesut\Desktop\kfz-insurance-risk-platform\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{846658C4-2EEF-4601-AC11-63087F5E43D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC82DB2-BFCB-478A-9A47-462C16E2DF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
   <si>
     <t>Zeiterfassung Abschlussprojekt — Mesut Karagöz</t>
   </si>
@@ -238,6 +238,36 @@
   </si>
   <si>
     <t>Validierung und Dokumentation</t>
+  </si>
+  <si>
+    <t>Geschäftsorientierte EDA gestartet und zentrale Portfoliokennzahlen analysiert</t>
+  </si>
+  <si>
+    <t>Schadenfrequenz nach Fahrer-, Fahrzeug- und Tarifmerkmalen analysiert</t>
+  </si>
+  <si>
+    <t>Schadenhöhenverteilung, Großschäden und beobachtete Pure Premium untersucht</t>
+  </si>
+  <si>
+    <t>Einfachen Exposure-gewichteten Poisson-Kontrollpunkt umgesetzt und Policy-Level-Prognosen erzeugt</t>
+  </si>
+  <si>
+    <t>PostgreSQL-Prediction-View und Power-BI-Anbindung validiert sowie End-to-End-Kette abgeschlossen</t>
+  </si>
+  <si>
+    <t>Explorative Datenanalyse</t>
+  </si>
+  <si>
+    <t>Risikoanalyse</t>
+  </si>
+  <si>
+    <t>Severity- und Pure-Premium-Analyse</t>
+  </si>
+  <si>
+    <t>Modell-Kontrollpunkt</t>
+  </si>
+  <si>
+    <t>End-to-End-Validierung</t>
   </si>
 </sst>
 </file>
@@ -439,12 +469,12 @@
     <xf numFmtId="165" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -721,74 +751,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="29"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1231,114 +1261,214 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="7"/>
-      <c r="B30" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="8"/>
+      <c r="A30" s="2">
+        <v>46258</v>
+      </c>
+      <c r="B30" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E30" s="5">
+        <v>5</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="7"/>
-      <c r="B31" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="8"/>
+      <c r="A31" s="2">
+        <v>46258</v>
+      </c>
+      <c r="B31" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" s="5">
+        <v>2</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="7"/>
-      <c r="B32" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="8"/>
+      <c r="A32" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B32" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="5">
+        <v>6</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="7"/>
-      <c r="B33" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="8"/>
+      <c r="A33" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B33" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E33" s="5">
+        <v>1</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="7"/>
-      <c r="B34" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="8"/>
+      <c r="A34" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B34" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E34" s="5">
+        <v>4</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="7"/>
-      <c r="B35" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="8"/>
+      <c r="A35" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B35" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E35" s="5">
+        <v>3</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="7"/>
-      <c r="B36" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="8"/>
+      <c r="A36" s="2">
+        <v>46261</v>
+      </c>
+      <c r="B36" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E36" s="5">
+        <v>5</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="7"/>
-      <c r="B37" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="8"/>
+      <c r="A37" s="2">
+        <v>46261</v>
+      </c>
+      <c r="B37" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E37" s="5">
+        <v>2</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="7"/>
-      <c r="B38" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="8"/>
+      <c r="A38" s="2">
+        <v>46262</v>
+      </c>
+      <c r="B38" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E38" s="5">
+        <v>4</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="7"/>
-      <c r="B39" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="8"/>
+      <c r="A39" s="2">
+        <v>46262</v>
+      </c>
+      <c r="B39" s="3">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E39" s="5">
+        <v>3</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="7"/>
@@ -4503,7 +4633,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4521,24 +4651,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
@@ -4664,15 +4794,15 @@
       </c>
       <c r="D9" s="21">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A9,Zeiterfassung!$C$11:$C$325,"Abschlussprojekt")</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E9" s="21">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A9,Zeiterfassung!$C$11:$C$325,"Bewerbungen")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F9" s="22">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -4798,36 +4928,36 @@
       </c>
       <c r="D15" s="25">
         <f>SUM(D5:D14)</f>
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="E15" s="25">
         <f>SUM(E5:E14)</f>
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="F15" s="25">
         <f>SUM(F5:F14)</f>
-        <v>70</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Complete Week 7 Power BI, subgroup diagnostics and documentation
</commit_message>
<xml_diff>
--- a/docs/Zeiterfassung_Abschlussprojekt.xlsx
+++ b/docs/Zeiterfassung_Abschlussprojekt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mesut\Desktop\kfz-insurance-risk-platform\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC82DB2-BFCB-478A-9A47-462C16E2DF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264AEAFF-00AF-49D4-861C-D8982820FACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="80">
   <si>
     <t>Zeiterfassung Abschlussprojekt — Mesut Karagöz</t>
   </si>
@@ -268,6 +268,15 @@
   </si>
   <si>
     <t>End-to-End-Validierung</t>
+  </si>
+  <si>
+    <t>Geschäftsorientierte EDA durchgeführt und zentrale Portfoliokennzahlen analysiert</t>
+  </si>
+  <si>
+    <t>Exposure-gewichteten Poisson-Kontrollpunkt entwickelt und Policy-Level-Prognosen erzeugt</t>
+  </si>
+  <si>
+    <t>Prognosen in PostgreSQL gespeichert und End-to-End-Kette bis Power BI validiert</t>
   </si>
 </sst>
 </file>
@@ -1471,114 +1480,214 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="7"/>
-      <c r="B40" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="8"/>
+      <c r="A40" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B40" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E40" s="5">
+        <v>5</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="7"/>
-      <c r="B41" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="8"/>
+      <c r="A41" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B41" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E41" s="5">
+        <v>2</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="7"/>
-      <c r="B42" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="8"/>
+      <c r="A42" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B42" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E42" s="5">
+        <v>4</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="7"/>
-      <c r="B43" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="8"/>
+      <c r="A43" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B43" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E43" s="5">
+        <v>3</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="7"/>
-      <c r="B44" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="8"/>
+      <c r="A44" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B44" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E44" s="5">
+        <v>4</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="7"/>
-      <c r="B45" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="8"/>
+      <c r="A45" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B45" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" s="5">
+        <v>3</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="7"/>
-      <c r="B46" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="8"/>
+      <c r="A46" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B46" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E46" s="5">
+        <v>5</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="7"/>
-      <c r="B47" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="8"/>
+      <c r="A47" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B47" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E47" s="5">
+        <v>2</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
-      <c r="B48" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="8"/>
+      <c r="A48" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B48" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E48" s="5">
+        <v>6</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="7"/>
-      <c r="B49" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="8"/>
+      <c r="A49" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B49" s="3">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E49" s="5">
+        <v>1</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="7"/>
@@ -4817,15 +4926,15 @@
       </c>
       <c r="D10" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A10,Zeiterfassung!$C$11:$C$325,"Abschlussprojekt")</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E10" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A10,Zeiterfassung!$C$11:$C$325,"Bewerbungen")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F10" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -4928,15 +5037,15 @@
       </c>
       <c r="D15" s="25">
         <f>SUM(D5:D14)</f>
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="E15" s="25">
         <f>SUM(E5:E14)</f>
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="F15" s="25">
         <f>SUM(F5:F14)</f>
-        <v>105</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Finalize Power BI dashboard and add dashboard assets
</commit_message>
<xml_diff>
--- a/docs/Zeiterfassung_Abschlussprojekt.xlsx
+++ b/docs/Zeiterfassung_Abschlussprojekt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mesut\Desktop\kfz-insurance-risk-platform\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264AEAFF-00AF-49D4-861C-D8982820FACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76F8EC3E-9293-4256-B6B2-A116646B1D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="99">
   <si>
     <t>Zeiterfassung Abschlussprojekt — Mesut Karagöz</t>
   </si>
@@ -277,6 +277,63 @@
   </si>
   <si>
     <t>Prognosen in PostgreSQL gespeichert und End-to-End-Kette bis Power BI validiert</t>
+  </si>
+  <si>
+    <t>Abschlussprojekt – Gemeinsamen Train-/Test-Split geprüft und Frequency-Modell weiterentwickelt</t>
+  </si>
+  <si>
+    <t>Bewerbungen – Stellensuche und Bewerbungsaktivitäten</t>
+  </si>
+  <si>
+    <t>Abschlussprojekt – Frequency-v2-Modell validiert, Deviance und Gini ausgewertet</t>
+  </si>
+  <si>
+    <t>Bewerbungen – Stellenrecherche und Bewerbungsunterlagen</t>
+  </si>
+  <si>
+    <t>Abschlussprojekt – Severity-v2-Modell, Cross-Validation und Regularisierung ausgewertet</t>
+  </si>
+  <si>
+    <t>Bewerbungen – Stellensuche, Bewerbungen und Nachverfolgung</t>
+  </si>
+  <si>
+    <t>Abschlussprojekt – Frequency und Severity zur Pure Premium kombiniert und Portfolio-Kalibrierung geprüft</t>
+  </si>
+  <si>
+    <t>Bewerbungen – Stellenrecherche und Bewerbungsaktivitäten</t>
+  </si>
+  <si>
+    <t>Abschlussprojekt – Finale Modelle versioniert, Policy-Level-Prognosen erstellt und PostgreSQL-Integration validiert</t>
+  </si>
+  <si>
+    <t>Split validiert, kein IDpol-Leakage</t>
+  </si>
+  <si>
+    <t>Stellen recherchiert und Bewerbungen geprüft</t>
+  </si>
+  <si>
+    <t>Frequency v2 als finales Modell festgelegt</t>
+  </si>
+  <si>
+    <t>Bewerbungsunterlagen angepasst</t>
+  </si>
+  <si>
+    <t>Severity v2 validiert, Modellgrenzen dokumentiert</t>
+  </si>
+  <si>
+    <t>Offene Bewerbungen geprüft und neue Stellen recherchiert</t>
+  </si>
+  <si>
+    <t>Pure Premium und Portfolioabweichungen validiert</t>
+  </si>
+  <si>
+    <t>Geeignete Stellen recherchiert und Bewerbungen bearbeitet</t>
+  </si>
+  <si>
+    <t>678.013 Prognosen erzeugt und PostgreSQL-Integration geprüft</t>
+  </si>
+  <si>
+    <t>Bewerbungsaktivitäten dokumentiert und nachverfolgt</t>
   </si>
 </sst>
 </file>
@@ -1690,114 +1747,214 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="7"/>
-      <c r="B50" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="8"/>
+      <c r="A50" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B50" s="3">
+        <f>IF(A50="","",WEEKNUM(A50,2))</f>
+        <v>37</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E50" s="5">
+        <v>4</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="7"/>
-      <c r="B51" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="8"/>
+      <c r="A51" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B51" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E51" s="5">
+        <v>3</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="7"/>
-      <c r="B52" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="8"/>
+      <c r="A52" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B52" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E52" s="5">
+        <v>5</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="7"/>
-      <c r="B53" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="8"/>
+      <c r="A53" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B53" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E53" s="5">
+        <v>2</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="7"/>
-      <c r="B54" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="8"/>
+      <c r="A54" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B54" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E54" s="5">
+        <v>5</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="7"/>
-      <c r="B55" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C55" s="8"/>
-      <c r="D55" s="8"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="8"/>
+      <c r="A55" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B55" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E55" s="5">
+        <v>2</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="7"/>
-      <c r="B56" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C56" s="8"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="8"/>
+      <c r="A56" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B56" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E56" s="5">
+        <v>6</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="7"/>
-      <c r="B57" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C57" s="8"/>
-      <c r="D57" s="8"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="8"/>
+      <c r="A57" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B57" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E57" s="5">
+        <v>1</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="7"/>
-      <c r="B58" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C58" s="8"/>
-      <c r="D58" s="8"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="8"/>
+      <c r="A58" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B58" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E58" s="5">
+        <v>5</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="7"/>
-      <c r="B59" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C59" s="8"/>
-      <c r="D59" s="8"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="8"/>
+      <c r="A59" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B59" s="3">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E59" s="5">
+        <v>2</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="7"/>
@@ -4949,15 +5106,15 @@
       </c>
       <c r="D11" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A11,Zeiterfassung!$C$11:$C$325,"Abschlussprojekt")</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E11" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A11,Zeiterfassung!$C$11:$C$325,"Bewerbungen")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F11" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -5037,15 +5194,15 @@
       </c>
       <c r="D15" s="25">
         <f>SUM(D5:D14)</f>
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="E15" s="25">
         <f>SUM(E5:E14)</f>
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="F15" s="25">
         <f>SUM(F5:F14)</f>
-        <v>140</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update Power BI, time tracking and final presentation
</commit_message>
<xml_diff>
--- a/docs/Zeiterfassung_Abschlussprojekt.xlsx
+++ b/docs/Zeiterfassung_Abschlussprojekt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mesut\Desktop\kfz-insurance-risk-platform\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76F8EC3E-9293-4256-B6B2-A116646B1D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8205EFA7-F3A7-44D0-9897-198DD8684AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="132">
   <si>
     <t>Zeiterfassung Abschlussprojekt — Mesut Karagöz</t>
   </si>
@@ -334,6 +334,105 @@
   </si>
   <si>
     <t>Bewerbungsaktivitäten dokumentiert und nachverfolgt</t>
+  </si>
+  <si>
+    <t>Tweedie-Ziel und geeignete Modellpopulation definiert sowie Train-Side-Modellwahl durchgeführt</t>
+  </si>
+  <si>
+    <t>Stellensuche und Bewerbungsaktivitäten</t>
+  </si>
+  <si>
+    <t>Tweedie-Modell validiert und Two-Stage mit Tweedie anhand Deviance, Gini und Portfolio-Kalibrierung verglichen</t>
+  </si>
+  <si>
+    <t>Bewerbungen vorbereitet und Bewerbungsunterlagen angepasst</t>
+  </si>
+  <si>
+    <t>Modell-Erklärbarkeit mit GLM-Koeffizienten, Permutation Importance sowie PDP- und ICE-Analysen durchgeführt</t>
+  </si>
+  <si>
+    <t>Stellensuche, Bewerbungen und Nachverfolgung</t>
+  </si>
+  <si>
+    <t>Risikosegmente und Risk Deciles erstellt sowie Business-Handlungsempfehlungen und Management-KPIs abgeleitet</t>
+  </si>
+  <si>
+    <t>Stellenrecherche und Bewerbungsaktivitäten</t>
+  </si>
+  <si>
+    <t>FastAPI auf finale Modelllogik angepasst, vier Endpunkte validiert, sechs Tests durchgeführt und Ergebnisse dokumentiert</t>
+  </si>
+  <si>
+    <t>Bewerbungsaktivitäten dokumentiert und offene Bewerbungen nachverfolgt</t>
+  </si>
+  <si>
+    <t>Tweedie-Challenger und Modellselektion</t>
+  </si>
+  <si>
+    <t>Geeignete Stellen recherchiert und Bewerbungen geprüft</t>
+  </si>
+  <si>
+    <t>Modellvergleich und finale Modellentscheidung</t>
+  </si>
+  <si>
+    <t>Explainability und Modellinterpretation</t>
+  </si>
+  <si>
+    <t>Offene Bewerbungen geprüft</t>
+  </si>
+  <si>
+    <t>Risk Segmentation und Decision Support</t>
+  </si>
+  <si>
+    <t>Neue Stellen recherchiert und Bewerbungen bearbeitet</t>
+  </si>
+  <si>
+    <t>API-Validierung, Tests und Wochenabschluss</t>
+  </si>
+  <si>
+    <t>Power-BI-Datenmodell, Datenquellen und zentrale KPI-Logik geprüft und final abgestimmt</t>
+  </si>
+  <si>
+    <t>Portfolio Overview und Risk Segmentation im Power-BI-Dashboard finalisiert</t>
+  </si>
+  <si>
+    <t>Bewerbungsunterlagen geprüft und Stellen recherchiert</t>
+  </si>
+  <si>
+    <t>Expected Loss, Pure Premium sowie Data Quality und Model Validation im Dashboard aufbereitet</t>
+  </si>
+  <si>
+    <t>Stellensuche und Nachverfolgung bestehender Bewerbungen</t>
+  </si>
+  <si>
+    <t>Subgruppen-Performance für Frequency, Severity und Tweedie ausgewertet und Responsible Use dokumentiert</t>
+  </si>
+  <si>
+    <t>Bewerbungen recherchiert und Bewerbungsunterlagen angepasst</t>
+  </si>
+  <si>
+    <t>README, Model Card, Data Dictionary, Data Quality Report und Architektur final geprüft sowie Projektkonsistenz kontrolliert</t>
+  </si>
+  <si>
+    <t>Bewerbungsaktivitäten dokumentiert und offene Bewerbungen geprüft</t>
+  </si>
+  <si>
+    <t>Power BI, Datenmodell und Exposure-basierte KPI-Logik</t>
+  </si>
+  <si>
+    <t>Geeignete Stellen recherchiert und offene Bewerbungen geprüft</t>
+  </si>
+  <si>
+    <t>Dashboard-Seiten, Risk Segments und Risk Deciles</t>
+  </si>
+  <si>
+    <t>Modellvergleich, DQ und Pipeline Monitoring</t>
+  </si>
+  <si>
+    <t>Alter, Region, Area und Density analysiert</t>
+  </si>
+  <si>
+    <t>Dokumentation, Consistency Check und Abschlussvorbereitung</t>
   </si>
 </sst>
 </file>
@@ -1957,224 +2056,424 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="7"/>
-      <c r="B60" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="8"/>
+      <c r="A60" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B60" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E60" s="5">
+        <v>5</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="7"/>
-      <c r="B61" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C61" s="8"/>
-      <c r="D61" s="8"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="8"/>
+      <c r="A61" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B61" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E61" s="5">
+        <v>2</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="7"/>
-      <c r="B62" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C62" s="8"/>
-      <c r="D62" s="8"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="8"/>
+      <c r="A62" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B62" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E62" s="5">
+        <v>5</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="7"/>
-      <c r="B63" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C63" s="8"/>
-      <c r="D63" s="8"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="8"/>
+      <c r="A63" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B63" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E63" s="5">
+        <v>2</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="7"/>
-      <c r="B64" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C64" s="8"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="8"/>
+      <c r="A64" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B64" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E64" s="5">
+        <v>5</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="7"/>
-      <c r="B65" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C65" s="8"/>
-      <c r="D65" s="8"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="8"/>
+      <c r="A65" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B65" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E65" s="5">
+        <v>2</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="7"/>
-      <c r="B66" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C66" s="8"/>
-      <c r="D66" s="8"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="8"/>
+      <c r="A66" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B66" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E66" s="5">
+        <v>5</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="7"/>
-      <c r="B67" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C67" s="8"/>
-      <c r="D67" s="8"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="8"/>
+      <c r="A67" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E67" s="5">
+        <v>2</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="7"/>
-      <c r="B68" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C68" s="8"/>
-      <c r="D68" s="8"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="8"/>
+      <c r="A68" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E68" s="5">
+        <v>4</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="7"/>
-      <c r="B69" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C69" s="8"/>
-      <c r="D69" s="8"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="8"/>
+      <c r="A69" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B69" s="3">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E69" s="5">
+        <v>3</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="7"/>
-      <c r="B70" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C70" s="8"/>
-      <c r="D70" s="8"/>
-      <c r="E70" s="9"/>
-      <c r="F70" s="8"/>
+      <c r="A70" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B70" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E70" s="5">
+        <v>5</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="7"/>
-      <c r="B71" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C71" s="8"/>
-      <c r="D71" s="8"/>
-      <c r="E71" s="9"/>
-      <c r="F71" s="8"/>
+      <c r="A71" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E71" s="5">
+        <v>2</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="7"/>
-      <c r="B72" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C72" s="8"/>
-      <c r="D72" s="8"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="8"/>
+      <c r="A72" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E72" s="5">
+        <v>5</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="7"/>
-      <c r="B73" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C73" s="8"/>
-      <c r="D73" s="8"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="8"/>
+      <c r="A73" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B73" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E73" s="5">
+        <v>2</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="7"/>
-      <c r="B74" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C74" s="8"/>
-      <c r="D74" s="8"/>
-      <c r="E74" s="9"/>
-      <c r="F74" s="8"/>
+      <c r="A74" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B74" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E74" s="5">
+        <v>5</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="7"/>
-      <c r="B75" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="9"/>
-      <c r="F75" s="8"/>
+      <c r="A75" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B75" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E75" s="5">
+        <v>2</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="7"/>
-      <c r="B76" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="9"/>
-      <c r="F76" s="8"/>
+      <c r="A76" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B76" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E76" s="5">
+        <v>5</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="7"/>
-      <c r="B77" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
-      <c r="E77" s="9"/>
-      <c r="F77" s="8"/>
+      <c r="A77" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B77" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E77" s="5">
+        <v>2</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="7"/>
-      <c r="B78" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="9"/>
-      <c r="F78" s="8"/>
+      <c r="A78" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B78" s="3">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="E78" s="5">
+        <v>5</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="7"/>
-      <c r="B79" s="3" t="str">
+      <c r="A79" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B79" s="3">
         <f t="shared" ref="B79:B142" si="6">IF(A79="","",WEEKNUM(A79,2))</f>
-        <v/>
-      </c>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="9"/>
-      <c r="F79" s="8"/>
+        <v>39</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E79" s="5">
+        <v>2</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="7"/>
@@ -5129,15 +5428,15 @@
       </c>
       <c r="D12" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A12,Zeiterfassung!$C$11:$C$325,"Abschlussprojekt")</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E12" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A12,Zeiterfassung!$C$11:$C$325,"Bewerbungen")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F12" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -5152,15 +5451,15 @@
       </c>
       <c r="D13" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A13,Zeiterfassung!$C$11:$C$325,"Abschlussprojekt")</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E13" s="13">
         <f>SUMIFS(Zeiterfassung!$E$11:$E$325,Zeiterfassung!$B$11:$B$325,$A13,Zeiterfassung!$C$11:$C$325,"Bewerbungen")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F13" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -5194,15 +5493,15 @@
       </c>
       <c r="D15" s="25">
         <f>SUM(D5:D14)</f>
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="E15" s="25">
         <f>SUM(E5:E14)</f>
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="F15" s="25">
         <f>SUM(F5:F14)</f>
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>